<commit_message>
Validaciones de editar y agregar producto
</commit_message>
<xml_diff>
--- a/mi-proyecto/docs/Ruta_Rec_Hu.xlsx
+++ b/mi-proyecto/docs/Ruta_Rec_Hu.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t xml:space="preserve">El usuario solo podra ingresar “Unidad de medida” o “Unidad agrupada” al momento de agregar P</t>
   </si>
@@ -38,6 +38,9 @@
   </si>
   <si>
     <t xml:space="preserve">La venta de un producto provoca una salidad en lotes usando FEFO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dificil</t>
   </si>
   <si>
     <t xml:space="preserve">Habra una tabala Dias que contendra la fecha del dia anterior, cuando el dia sea menor que el dia 
@@ -60,6 +63,9 @@
   <si>
     <t xml:space="preserve">El filtor de A.P de ve mostar las unidades de medida o {id, nombre, marca} dependiendo de la 
 Opcion ejegida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Podra filtrar P por codigo, nombre y marca</t>
   </si>
 </sst>
 </file>
@@ -74,7 +80,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -96,7 +101,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -154,7 +158,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -335,10 +339,13 @@
       <c r="B6" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="C6" s="0" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0</v>
@@ -346,7 +353,7 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0</v>
@@ -354,7 +361,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0</v>
@@ -362,7 +369,7 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0</v>
@@ -370,7 +377,7 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0</v>
@@ -378,13 +385,19 @@
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="C13" s="3"/>
     </row>
   </sheetData>

</xml_diff>